<commit_message>
fix: Remove too specific prefix
</commit_message>
<xml_diff>
--- a/assets/resources/invoice/invoice_patients_template.xlsx
+++ b/assets/resources/invoice/invoice_patients_template.xlsx
@@ -21,9 +21,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
-  <si>
-    <t xml:space="preserve">NENT N</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="17">
+  <si>
+    <t xml:space="preserve">NENT</t>
   </si>
   <si>
     <t xml:space="preserve">Einzelrechnung</t>
@@ -69,9 +69,6 @@
   </si>
   <si>
     <t xml:space="preserve">Zusammenfassung</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NENT</t>
   </si>
   <si>
     <t xml:space="preserve">Ref.-Nr.</t>
@@ -400,6 +397,9 @@
       <c r="F1" s="2"/>
       <c r="G1" s="2"/>
     </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0"/>
+    </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
         <v>3</v>
@@ -508,10 +508,10 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>16</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>17</v>
       </c>
       <c r="D3" s="4" t="s">
         <v>13</v>

</xml_diff>